<commit_message>
Exam Excel : advance on-progress
</commit_message>
<xml_diff>
--- a/Exam/Excel/advanced_assessment_project/Master_Customer_Profile.xlsx
+++ b/Exam/Excel/advanced_assessment_project/Master_Customer_Profile.xlsx
@@ -8,51 +8,187 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\Project\Data-Analyst\Exam\Excel\advanced_assessment_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{173CCBA6-71EC-4D9B-9588-C0713B3D8F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C35ADC5-55D7-4C08-99A0-1A5A098C500E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{3C5588B9-965A-4528-9C30-1A6079391BAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Master_Customer_Profile" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>Cust_ID,Raw_Name,Raw_Phone,Region,City,Join_Date,Membership_Tier</t>
-  </si>
-  <si>
-    <t>CUST-001,  Ahmad  Fauzi ,081234567890,Jawa Barat,Bandung,2022-01-15,VIP</t>
-  </si>
-  <si>
-    <t>CUST-002,Siti Nurhaliza  ,+628189876543,DKI Jakarta,Jakarta Selatan,2023-03-20,Gold</t>
-  </si>
-  <si>
-    <t>CUST-003,  budi santoso,6285611223344,Jawa Tengah,Semarang,2021-11-05,Platinum</t>
-  </si>
-  <si>
-    <t>CUST-004,DEWI LESTARI,087855443322,Jawa Timur,Surabaya,2023-08-12,Silver</t>
-  </si>
-  <si>
-    <t>CUST-005, hendra wijaya  ,+62 813 9988 7766,DKI Jakarta,Jakarta Barat,2022-06-30,Gold</t>
-  </si>
-  <si>
-    <t>CUST-006,Rina  Anggraini ,081122334455,Banten,Tangerang,2024-01-10,Silver</t>
-  </si>
-  <si>
-    <t>CUST-007, EKO PRASETYO ,628170099887,DI Yogyakarta,Yogyakarta,2020-04-18,Platinum</t>
-  </si>
-  <si>
-    <t>CUST-008,Maya  Indah  Sari,085211447788,Sumatera Utara,Medan,2023-05-22,Gold</t>
-  </si>
-  <si>
-    <t>CUST-009,  rizky hidayat ,+62 819 3322 1100,Sulawesi Selatan,Makassar,2022-09-14,Silver</t>
-  </si>
-  <si>
-    <t>CUST-010,VALENTINA ROSI,081377665544,Bali,Denpasar,2021-12-01,VIP</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="51">
+  <si>
+    <t>Cust_ID</t>
+  </si>
+  <si>
+    <t>Raw_Name</t>
+  </si>
+  <si>
+    <t>Raw_Phone</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Join_Date</t>
+  </si>
+  <si>
+    <t>Membership_Tier</t>
+  </si>
+  <si>
+    <t>CUST-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Ahmad  Fauzi </t>
+  </si>
+  <si>
+    <t>Jawa Barat</t>
+  </si>
+  <si>
+    <t>Bandung</t>
+  </si>
+  <si>
+    <t>VIP</t>
+  </si>
+  <si>
+    <t>CUST-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siti Nurhaliza  </t>
+  </si>
+  <si>
+    <t>DKI Jakarta</t>
+  </si>
+  <si>
+    <t>Jakarta Selatan</t>
+  </si>
+  <si>
+    <t>Gold</t>
+  </si>
+  <si>
+    <t>CUST-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  budi santoso</t>
+  </si>
+  <si>
+    <t>Jawa Tengah</t>
+  </si>
+  <si>
+    <t>Semarang</t>
+  </si>
+  <si>
+    <t>Platinum</t>
+  </si>
+  <si>
+    <t>CUST-004</t>
+  </si>
+  <si>
+    <t>DEWI LESTARI</t>
+  </si>
+  <si>
+    <t>Jawa Timur</t>
+  </si>
+  <si>
+    <t>Surabaya</t>
+  </si>
+  <si>
+    <t>Silver</t>
+  </si>
+  <si>
+    <t>CUST-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> hendra wijaya  </t>
+  </si>
+  <si>
+    <t>Jakarta Barat</t>
+  </si>
+  <si>
+    <t>CUST-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rina  Anggraini </t>
+  </si>
+  <si>
+    <t>Banten</t>
+  </si>
+  <si>
+    <t>Tangerang</t>
+  </si>
+  <si>
+    <t>CUST-007</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> EKO PRASETYO </t>
+  </si>
+  <si>
+    <t>DI Yogyakarta</t>
+  </si>
+  <si>
+    <t>Yogyakarta</t>
+  </si>
+  <si>
+    <t>CUST-008</t>
+  </si>
+  <si>
+    <t>Maya  Indah  Sari</t>
+  </si>
+  <si>
+    <t>Sumatera Utara</t>
+  </si>
+  <si>
+    <t>Medan</t>
+  </si>
+  <si>
+    <t>CUST-009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  rizky hidayat </t>
+  </si>
+  <si>
+    <t>+62 819 3322 1100</t>
+  </si>
+  <si>
+    <t>Sulawesi Selatan</t>
+  </si>
+  <si>
+    <t>Makassar</t>
+  </si>
+  <si>
+    <t>CUST-010</t>
+  </si>
+  <si>
+    <t>VALENTINA ROSI</t>
+  </si>
+  <si>
+    <t>Bali</t>
+  </si>
+  <si>
+    <t>Denpasar</t>
   </si>
 </sst>
 </file>
@@ -195,7 +331,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -375,8 +511,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -491,6 +633,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -536,8 +693,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -594,6 +754,28 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Raw_Transactions_2024"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="2">
+          <cell r="O2" t="str">
+            <v>8189876543</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -913,62 +1095,269 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95B2CEDF-7BD6-4DDD-91E5-297F8E61AF97}">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1">
+        <v>81234567890</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2">
+        <v>44576</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="1">
+        <v>628189876543</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="2">
+        <v>45005</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1">
+        <v>6285611223344</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="2">
+        <v>44505</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="1">
+        <v>87855443322</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="2">
+        <v>45150</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>5</v>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="1" t="str">
+        <f>[1]Raw_Transactions_2024!$O$2</f>
+        <v>8189876543</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="2">
+        <v>44742</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>6</v>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="1">
+        <v>81122334455</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="2">
+        <v>45301</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="1">
+        <v>628170099887</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="2">
+        <v>43939</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>8</v>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="1">
+        <v>85211447788</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="2">
+        <v>45068</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>9</v>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="2">
+        <v>44818</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>10</v>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="1">
+        <v>81377665544</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" s="2">
+        <v>44531</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>